<commit_message>
Align public content with document contract
</commit_message>
<xml_diff>
--- a/public/requirements-definition-template-ja.xlsx
+++ b/public/requirements-definition-template-ja.xlsx
@@ -33,12 +33,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="103">
-  <si>
-    <t xml:space="preserve">要件定義書テンプレート｜項目概要</t>
-  </si>
-  <si>
-    <t xml:space="preserve">製品が生成する要件定義書と同じ列順です。案件情報を入力し、未決事項は関係者レビューで確認してください。</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="95">
+  <si>
+    <t xml:space="preserve">項目概要｜無料テンプレート</t>
+  </si>
+  <si>
+    <t xml:space="preserve">製品が生成する正式構造です。案件固有の内容を記入し、関係者レビューを行ってください。</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -50,7 +50,7 @@
     <t xml:space="preserve">内容</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜スコープ定義</t>
+    <t xml:space="preserve">スコープ定義｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">区分</t>
@@ -62,7 +62,7 @@
     <t xml:space="preserve">説明</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜業務要件</t>
+    <t xml:space="preserve">業務要件｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">業務</t>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">要件</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜機能要件一覧</t>
+    <t xml:space="preserve">機能要件一覧｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">機能名</t>
@@ -89,14 +89,14 @@
     <t xml:space="preserve">優先度</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜画面一覧</t>
+    <t xml:space="preserve">画面一覧｜無料テンプレート</t>
   </si>
   <si>
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF0F172A"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
@@ -105,9 +105,9 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF0F172A"/>
-        <rFont val="Yu Gothic"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -121,13 +121,13 @@
     <t xml:space="preserve">主な機能</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜画面概要</t>
+    <t xml:space="preserve">画面概要｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">利用者</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜権限一覧</t>
+    <t xml:space="preserve">権限一覧｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">ロール名</t>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">利用可能機能</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜データ項目定義</t>
+    <t xml:space="preserve">データ項目定義｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">エンティティ名</t>
@@ -153,14 +153,14 @@
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">要件定義書テンプレート｜外部連携・</t>
+      <t xml:space="preserve">外部連携・</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="16"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="Yu Gothic"/>
+        <rFont val="Calibri"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -174,16 +174,16 @@
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">一覧</t>
+      <t xml:space="preserve">一覧｜無料テンプレート</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF0F172A"/>
-        <rFont val="Yu Gothic"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -192,8 +192,8 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF0F172A"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
@@ -210,13 +210,13 @@
     <t xml:space="preserve">業務説明</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜非機能要件</t>
+    <t xml:space="preserve">非機能要件｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">分類</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜業務フロー</t>
+    <t xml:space="preserve">業務フロー｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">ステップ</t>
@@ -225,16 +225,16 @@
     <t xml:space="preserve">担当</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜課題・リスク一覧</t>
+    <t xml:space="preserve">課題・リスク一覧｜無料テンプレート</t>
   </si>
   <si>
     <t xml:space="preserve">影響</t>
   </si>
   <si>
-    <t xml:space="preserve">要件定義書テンプレート｜レビュー・チェックリスト</t>
-  </si>
-  <si>
-    <t xml:space="preserve">状態はプルダウンで選択できます。未確認・確認中を残したまま承認せず、確認者、確認日、備考を記録してください。</t>
+    <t xml:space="preserve">レビュー・チェックリスト｜無料テンプレート附属</t>
+  </si>
+  <si>
+    <t xml:space="preserve">このシートは製品生成結果には含まれないレビュー補助資料です。状態、確認者、確認日、備考を記録してください。</t>
   </si>
   <si>
     <t xml:space="preserve">チェック項目</t>
@@ -252,7 +252,7 @@
     <t xml:space="preserve">備考</t>
   </si>
   <si>
-    <t xml:space="preserve">目的・範囲</t>
+    <t xml:space="preserve">目的・背景</t>
   </si>
   <si>
     <t xml:space="preserve">解決する業務課題と期待効果が合意されている</t>
@@ -261,64 +261,94 @@
     <t xml:space="preserve">未確認</t>
   </si>
   <si>
+    <t xml:space="preserve">スコープ</t>
+  </si>
+  <si>
     <t xml:space="preserve">対象範囲と対象外範囲が明記されている</t>
   </si>
   <si>
-    <t xml:space="preserve">前提条件と制約に責任者がいる</t>
-  </si>
-  <si>
-    <t xml:space="preserve">機能・データ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">各機能に利用者と受入条件がある</t>
-  </si>
-  <si>
-    <t xml:space="preserve">主要データの作成・更新・削除権限が明確である</t>
-  </si>
-  <si>
-    <t xml:space="preserve">例外処理とエラー時の運用が定義されている</t>
-  </si>
-  <si>
-    <t xml:space="preserve">非機能・運用</t>
-  </si>
-  <si>
-    <t xml:space="preserve">性能値と測定条件が具体的である</t>
-  </si>
-  <si>
-    <t xml:space="preserve">可用性、バックアップ、復旧目標が確認済みである</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ログ、監査、保守、問い合わせ体制が整理されている</t>
-  </si>
-  <si>
-    <t xml:space="preserve">連携・移行</t>
-  </si>
-  <si>
-    <t xml:space="preserve">外部システムの責任分界点が明確である</t>
-  </si>
-  <si>
-    <t xml:space="preserve">連携頻度、形式、失敗時の再処理が定義されている</t>
-  </si>
-  <si>
-    <t xml:space="preserve">移行対象、品質確認、切戻し方法がある</t>
-  </si>
-  <si>
-    <t xml:space="preserve">レビュー・合意</t>
-  </si>
-  <si>
-    <t xml:space="preserve">未決事項に期限と責任者が設定されている</t>
-  </si>
-  <si>
-    <t xml:space="preserve">業務・開発・運用・セキュリティがレビューした</t>
-  </si>
-  <si>
-    <t xml:space="preserve">承認版と変更管理方法が共有されている</t>
-  </si>
-  <si>
-    <t xml:space="preserve">要件定義書テンプレート｜記入例</t>
-  </si>
-  <si>
-    <t xml:space="preserve">架空の受注・請求管理プロジェクトの記入例です。そのまま実際の案件要件として使用せず、必ず案件関係者が確認してください。</t>
+    <t xml:space="preserve">業務要件</t>
+  </si>
+  <si>
+    <t xml:space="preserve">対象業務と例外時の運用が確認されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">機能要件</t>
+  </si>
+  <si>
+    <t xml:space="preserve">利用者、操作、対象データ、期待結果が判定できる</t>
+  </si>
+  <si>
+    <t xml:space="preserve">非機能要件</t>
+  </si>
+  <si>
+    <t xml:space="preserve">性能、可用性、セキュリティの条件が測定可能である</t>
+  </si>
+  <si>
+    <t xml:space="preserve">役割・権限</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ロールごとの参照・更新範囲が確認されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">画面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">主要画面の目的と利用者が整理されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">データ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">主要データ項目と保持方針が確認されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">外部連携</t>
+  </si>
+  <si>
+    <t xml:space="preserve">連携先、方式、頻度、異常時の扱いが確認されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">データ移行</t>
+  </si>
+  <si>
+    <t xml:space="preserve">移行対象、品質確認、切替手順が確認されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">運用</t>
+  </si>
+  <si>
+    <t xml:space="preserve">監視、バックアップ、問い合わせ対応が確認されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">リスク</t>
+  </si>
+  <si>
+    <t xml:space="preserve">主要リスクの影響と対応方針が記録されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">未決事項</t>
+  </si>
+  <si>
+    <t xml:space="preserve">未決事項ごとに責任者と期限が設定されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">レビュー</t>
+  </si>
+  <si>
+    <t xml:space="preserve">業務責任者とシステム責任者が確認している</t>
+  </si>
+  <si>
+    <t xml:space="preserve">移管</t>
+  </si>
+  <si>
+    <t xml:space="preserve">基本設計へ引き継ぐ前提と制約が整理されている</t>
+  </si>
+  <si>
+    <t xml:space="preserve">記入例｜無料テンプレート附属</t>
+  </si>
+  <si>
+    <t xml:space="preserve">受注・請求管理を題材にした架空例です。実案件の要件としてそのまま利用できません。</t>
   </si>
   <si>
     <t xml:space="preserve">記入例</t>
@@ -330,153 +360,35 @@
     <t xml:space="preserve">項目概要</t>
   </si>
   <si>
-    <t xml:space="preserve">見積・受注・請求情報を一元管理し、転記作業を削減する</t>
+    <t xml:space="preserve">受注から請求までを一元管理し、手作業の転記を減らす</t>
+  </si>
+  <si>
+    <t xml:space="preserve">業務責任者が目的と効果を確認する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">確認中</t>
+  </si>
+  <si>
+    <t xml:space="preserve">架空例</t>
+  </si>
+  <si>
+    <t xml:space="preserve">スコープ定義</t>
   </si>
   <si>
     <r>
       <rPr>
         <sz val="10"/>
+        <color rgb="FF1E293B"/>
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">月間転記件数を現状比</t>
+      <t xml:space="preserve">見積、受注、請求、会計</t>
     </r>
     <r>
       <rPr>
         <sz val="10"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">削減</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">確認済</t>
-  </si>
-  <si>
-    <t xml:space="preserve">架空例</t>
-  </si>
-  <si>
-    <t xml:space="preserve">スコープ定義</t>
-  </si>
-  <si>
-    <t xml:space="preserve">見積作成、受注登録、請求書発行、取引先管理</t>
-  </si>
-  <si>
-    <t xml:space="preserve">対象外は会計仕訳登録と倉庫在庫実査</t>
-  </si>
-  <si>
-    <t xml:space="preserve">機能要件一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">受注検索</t>
-  </si>
-  <si>
-    <t xml:space="preserve">担当者は取引先、期間、状態で受注を検索できる</t>
-  </si>
-  <si>
-    <t xml:space="preserve">指定条件と検索結果が一致する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">確認中</t>
-  </si>
-  <si>
-    <t xml:space="preserve">権限一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経理担当</t>
-  </si>
-  <si>
-    <t xml:space="preserve">請求確定、請求書出力、入金状態更新を利用可能とする</t>
-  </si>
-  <si>
-    <t xml:space="preserve">営業担当は請求確定できない</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">外部連携</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/API</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">一覧</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">会計</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CSV</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">確定済み請求データを毎日</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時に</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Yu Gothic"/>
+        <color rgb="FF1E293B"/>
+        <rFont val="Calibri"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -485,17 +397,15 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <color rgb="FF1E293B"/>
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">出力する</t>
+      <t xml:space="preserve">連携</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">失敗時は経理担当へ通知し再出力可能</t>
-  </si>
-  <si>
-    <t xml:space="preserve">非機能要件</t>
+    <t xml:space="preserve">対象外業務も合わせて合意する</t>
   </si>
   <si>
     <t xml:space="preserve">性能</t>
@@ -504,6 +414,7 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <color rgb="FF1E293B"/>
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
@@ -512,7 +423,8 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <rFont val="Yu Gothic"/>
+        <color rgb="FF1E293B"/>
+        <rFont val="Calibri"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
@@ -521,6 +433,7 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <color rgb="FF1E293B"/>
         <rFont val="Linux Libertine G"/>
         <family val="2"/>
       </rPr>
@@ -528,75 +441,16 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">同時利用</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">名の条件で測定</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">課題・リスク一覧</t>
-  </si>
-  <si>
-    <t xml:space="preserve">未決事項</t>
-  </si>
-  <si>
-    <t xml:space="preserve">旧システムから移行する請求履歴の期間</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">業務責任者が</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Linux Libertine G"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">月末までに決定</t>
-    </r>
+    <t xml:space="preserve">計測条件と対象画面を決める</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -634,22 +488,28 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF475569"/>
+      <color rgb="FF9A3412"/>
       <name val="Linux Libertine G"/>
       <family val="2"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF0F172A"/>
-      <name val="Yu Gothic"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Linux Libertine G"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
-      <color rgb="FF0F172A"/>
+      <color rgb="FF1E293B"/>
       <name val="Linux Libertine G"/>
       <family val="2"/>
     </font>
@@ -657,20 +517,16 @@
       <b val="true"/>
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Yu Gothic"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Yu Gothic"/>
+      <color rgb="FF1E293B"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Linux Libertine G"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -683,23 +539,23 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0F172A"/>
-        <bgColor rgb="FF000000"/>
+        <bgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF7E6"/>
+        <fgColor rgb="FFFFF7ED"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF59E0B"/>
-        <bgColor rgb="FFFFCC00"/>
+        <fgColor rgb="FFD97706"/>
+        <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -719,6 +575,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -752,7 +623,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -766,23 +637,19 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -797,6 +664,9 @@
   </cellStyles>
   <dxfs count="2">
     <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFEE2E2"/>
@@ -804,6 +674,9 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFEF3C7"/>
@@ -821,7 +694,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF991B1B"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -830,9 +703,9 @@
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF92400E"/>
       <rgbColor rgb="FFFEF3C7"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFE2E8F0"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -848,7 +721,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFF7E6"/>
+      <rgbColor rgb="FFFFF7ED"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -857,18 +730,18 @@
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFF59E0B"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF475569"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFD97706"/>
+      <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF0F172A"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF9A3412"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF1E293B"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1048,37 +921,29 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1089,65 +954,105 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1169,43 +1074,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1219,77 +1112,125 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1311,43 +1252,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1361,77 +1290,125 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1453,44 +1430,32 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1504,77 +1469,125 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1596,56 +1609,34 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>36</v>
       </c>
@@ -1665,7 +1656,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>49</v>
       </c>
@@ -1676,211 +1667,251 @@
         <v>51</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="E10" s="6"/>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="E16" s="6"/>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:C200">
+  <conditionalFormatting sqref="C5:C19">
     <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="未確認" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("未確認",C5)))</formula>
     </cfRule>
@@ -1889,7 +1920,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C200" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C19" type="list">
       <formula1>"未確認,確認中,確認済,対象外"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1909,54 +1940,34 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>80</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>36</v>
       </c>
@@ -1964,10 +1975,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>45</v>
@@ -1976,217 +1987,201 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" s="6" t="s">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="C5" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="C6" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="E8" s="6" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="F7" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2194,7 +2189,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E100" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E7" type="list">
       <formula1>"未確認,確認中,確認済,対象外"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2214,43 +2209,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2264,77 +2247,125 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2356,43 +2387,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2406,77 +2425,125 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2498,50 +2565,34 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2558,101 +2609,151 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
     </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E200" type="list">
-      <formula1>"高,中,低"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2668,49 +2769,32 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2727,89 +2811,145 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2831,43 +2971,31 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -2881,77 +3009,125 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2973,36 +3149,28 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3013,65 +3181,105 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3093,43 +3301,30 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="25.07"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3143,77 +3338,125 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3235,55 +3478,35 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="10.359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="21.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="45.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="25.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40.58"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3303,7 +3526,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -3311,7 +3534,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -3319,7 +3542,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -3327,7 +3550,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -3335,7 +3558,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -3343,7 +3566,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -3351,7 +3574,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -3359,7 +3582,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -3367,7 +3590,7 @@
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -3375,7 +3598,7 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -3383,7 +3606,7 @@
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -3391,13 +3614,77 @@
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="38" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>